<commit_message>
Segundo entregable: alinear actividad d) al Plan de Trabajo institucional v2 (firma espectral)
Anexo 3 reescrito con el Plan de Trabajo Detallado - Actualizacion N° 01,
Version 2 (16/10/2026) como documento rector: equipo base, cronograma
12/10-18/11/2026, EDT E6.1-E6.10, hitos H6g/H7b/H7c, riesgos R04/R05,
items adaptados del indice R00 y observaciones OE-14 a OE-16. Informe
principal (antecedentes, 4.3, conclusiones y recomendaciones), Anexo 2,
Anexo 4 y PDF consolidado actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J7Vxm47PRQCoCe3ph58u2J
</commit_message>
<xml_diff>
--- a/entregables/2do_entregable_OS4062/05_Anexo_4_Matrices_de_Seguimiento.xlsx
+++ b/entregables/2do_entregable_OS4062/05_Anexo_4_Matrices_de_Seguimiento.xlsx
@@ -23,9 +23,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Distritos'!$A$8:$N$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Situacion_predial'!$A$8:$N$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Obs_Suelos_E2'!$A$8:$G$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Obs_E6_Ecosistemas'!$A$8:$E$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Obs_E6_Ecosistemas'!$A$8:$E$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Obs_E6_Material_vegetal'!$A$8:$E$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Medios_verificadores'!$A$8:$E$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Medios_verificadores'!$A$8:$E$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19082,7 +19082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19223,22 +19223,22 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Plan v2.0, 10.1; Plan Detallado</t>
+          <t>Informe E6, ficha técnica y 9.2</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>El plan v2.0 cierra el E6 el 18/12/2026 y cita registro del Perfil en enero de 2027 (10.1) y en marzo de 2027 (sustento); el Plan Detallado fija la redacción final al 18/11/2026.</t>
+          <t>El informe cita como referencia metodológica el «E6 v2.0 sin parcelas» y toma de él las clases del IC; el plan institucional v2 dejó sin efecto esa modalidad y su programación al 18/12/2026.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Homologar fechas y horizonte en ambos documentos.</t>
+          <t>Citar como referencia el Plan de Trabajo institucional v2 y la Nota Técnica N° 002-2026; mantener el criterio del IC como propio del E6; fecha de redacción final 18/11/2026.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente (informe final)</t>
         </is>
       </c>
     </row>
@@ -19304,22 +19304,22 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>Informe E6, 9.6, 10.8 y 11</t>
+          <t>Informe E6, 9.6, 10.8 y 11; plan v2, 7.2</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>Validación ciega de 567 puntos y matriz de confusión no ejecutadas; el plan v2.0 comprometió exactitud global ≥ 85 %.</t>
+          <t>Matriz de confusión formal (≈ 600 puntos ciegos), TAU y estructura vertical no ejecutadas; el plan institucional las traslada al estudio definitivo.</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>Ejecutar la validación o declararla formalmente como vacío aceptado por SESDI.</t>
+          <t>Declararlas en el informe final como vacíos trasladados al estudio definitivo y someterlas a la conformidad de IN/SESDI (H7b).</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Encauzada por el plan v2; pendiente de conformidad</t>
         </is>
       </c>
     </row>
@@ -19336,12 +19336,12 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>El estrato de matorral andino bajo umbral tiene 10 de 20 parcelas requeridas (error 21.1 %).</t>
+          <t>El estrato de matorral andino bajo umbral tiene 10 de 20 lecturas requeridas (error 21.1 %).</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Densificar el estrato hasta cumplir el error de 15 %.</t>
+          <t>Densificar la lectura del estrato sobre el ráster de 1 m hasta el error de 15 %, o declarar la limitación.</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -19385,22 +19385,22 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Informe E6, 10.9; Plan Detallado</t>
+          <t>Informe E6, 10.9; plan v2, 1.4 d) y Tabla 8</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Coexisten tres criterios de brecha: areal del E6 (8,341.82 ha), media del bloque de los volúmenes DT y media por ecosistema propuesta en el Plan Detallado.</t>
+          <t>Coexisten tres criterios de brecha: areal del E6 (8,341.82 ha), media del bloque de los volúmenes DT (7,637.14 ha en 50 bloques) y media del MSAVI por ecosistema con umbral por ecosistema que propone el plan institucional.</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Adoptar por decisión de SESDI un criterio único para los 117 bloques.</t>
+          <t>Adoptar el criterio único con la aprobación del plan institucional y recalcular el indicador de los 117 bloques.</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente (decisión de SESDI)</t>
         </is>
       </c>
     </row>
@@ -19449,7 +19449,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Completar con consulta Delphi y verificar contra el anexo oficial del decreto.</t>
+          <t>Completar con consulta a especialistas y verificar contra el anexo oficial del decreto.</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -19493,17 +19493,17 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Plan v2.0, 12; hito H7b</t>
+          <t>Plan v2, Tabla 5 (H7b)</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>No se ha emitido el memorando de SESDI que acepte la adecuación metodológica.</t>
+          <t>No se ha emitido la conformidad de IN/SESDI sobre la metodología de firma espectral y los ítems adaptados del índice R00.</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Emitir el memorando de conformidad de la adecuación.</t>
+          <t>Emitir la conformidad sobre la base de la Nota Técnica N° 002-2026 (riesgo R04).</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -19513,21 +19513,102 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="19" t="n"/>
-      <c r="C22" s="19" t="n"/>
-      <c r="D22" s="19" t="n"/>
-      <c r="E22" s="19" t="n"/>
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>OE-14</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Plan v2, Tablas 4 y 12; matrices del plan</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>El avance del E6 figura como 39 % en el plan (corte 08/10/2026) y como 82.3 % en la hoja de avance de las matrices; los diez componentes registran avances distintos.</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Homologar el avance del E6 al mismo corte en el plan y en sus matrices.</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="n"/>
-      <c r="B23" s="19" t="n"/>
-      <c r="C23" s="19" t="n"/>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="19" t="n"/>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>OE-15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Informe E6, 7.1</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>El informe deja «por designar» a especialistas de flora, viveros, GdR y social; el plan institucional fija un equipo base sin contratación de personal.</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Alinear la nota del equipo al plan v2 y asignar la oferta de viveros según la reasignación de funciones (R05).</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>OE-16</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Informe E6, adecuación de ítems 9.5 y 10.7</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>El informe presenta las parcelas virtuales como unidad de muestreo; el plan institucional define el píxel de 1 m como unidad de análisis.</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Presentar las parcelas virtuales como resumen estadístico de la cobertura clasificada, conforme a la hoja «E6_Firma_Espectral».</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="n"/>
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="n"/>
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="19" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A8:E21"/>
+  <autoFilter ref="A8:E24"/>
   <mergeCells count="6">
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
@@ -19633,7 +19714,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Insumo OS 1147</t>
+          <t>Insumo OS 1147; plan v2, E6.6</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -19643,12 +19724,12 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Recalcular para los 117 bloques con las densidades, la mezcla y la reposición del E10 (hoja 16).</t>
+          <t>Calcular la demanda de los 117 bloques en el E10 con las densidades, la mezcla y la reposición (hoja 16), conforme al plan institucional.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente (E10)</t>
         </is>
       </c>
     </row>
@@ -19714,17 +19795,17 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>E6, fase 6</t>
+          <t>Informe E6, 9.7; plan v2, E6.7</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>El censo remoto de viveros (encuesta KoboToolbox y verificación en imágenes) no se ha ejecutado.</t>
+          <t>El censo remoto de viveros (encuesta y verificación en imágenes) no se ha ejecutado.</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Ejecutar el censo y calcular la oferta efectiva por especie.</t>
+          <t>Ejecutar el censo con el equipo base y calcular la oferta efectiva por especie antes del 18/11/2026.</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -19741,22 +19822,22 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Plan Detallado</t>
+          <t>Plan v2, 1.4 c) y R05</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Plaza de Especialista en Infraestructura Rural para la Producción (viveros) desierta.</t>
+          <t>Plaza de Especialista en Infraestructura Rural para la Producción (viveros) desierta y sin asignación presupuestal.</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Reasignar formalmente las funciones antes del 23/10/2026.</t>
+          <t>Formalizar la reasignación de funciones entre ESUS, EIV y EIM antes del 23/10/2026.</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente al corte de información del plan (16/10/2026)</t>
         </is>
       </c>
     </row>
@@ -19768,7 +19849,7 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>E6, 9.7</t>
+          <t>Plan v2, E6.7</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
@@ -19805,7 +19886,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Conciliar una lista única por piso, ecosistema y grupo de suelos.</t>
+          <t>Conciliar una lista única por piso, ecosistema y grupo de suelos para la entrega H7c.</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -19822,7 +19903,7 @@
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>E6, Tabla 15</t>
+          <t>Informe E6, Tabla 15</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
@@ -19875,7 +19956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20421,7 +20502,7 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>Plan de Trabajo Detallado, Actualización N° 02</t>
+          <t>Plan de Trabajo Detallado, Actualización N° 01, Versión 2 (documento rector del E6 por firma espectral)</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
@@ -20448,7 +20529,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Matrices del Plan de Trabajo (presupuesto ajustado)</t>
+          <t>Matrices del Plan de Trabajo (presupuesto ajustado; hoja «E6_Firma_Espectral»)</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
@@ -20475,7 +20556,7 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>E6 v2.0 «In house» (original)</t>
+          <t>E6 v2.0 «In house» (original; antecedente)</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
@@ -20610,7 +20691,7 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Informe E6 – versión para revisión de SESDI</t>
+          <t>Clasificación no supervisada de tomas S2DR4 (resultados y LEEME)</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -20620,12 +20701,12 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>1NfYjSV3QXI3uA4eHsMNQNTw9vdY5RdDA</t>
+          <t>1oZ-PLyuw4QyIBe-fupK3j7lQY_DE48J8; 1NRGviLNkpnvfyrLfv3dVNZms4w3SbfuS</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>13–14/10/2026</t>
         </is>
       </c>
     </row>
@@ -20637,7 +20718,7 @@
       </c>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>Matrices del diagnóstico del ecosistema (E6)</t>
+          <t>Informe E6 – versión para revisión de SESDI</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
@@ -20647,7 +20728,7 @@
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>1Uie1il6FeHI4SD8QhKXsfDof7cm4NF8J</t>
+          <t>1NfYjSV3QXI3uA4eHsMNQNTw9vdY5RdDA</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -20664,31 +20745,51 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
+          <t>Matrices del diagnóstico del ecosistema (E6)</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>1Uie1il6FeHI4SD8QhKXsfDof7cm4NF8J</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>d)</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
           <t>Fuentes semilleras de los Bosques Secos (referencia)</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>Google Drive</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>1hS8QlbTu_Ks05061BV4FAbAqbfUpikzy</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="E36" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="19" t="n"/>
-      <c r="B36" s="19" t="n"/>
-      <c r="C36" s="19" t="n"/>
-      <c r="D36" s="19" t="n"/>
-      <c r="E36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="19" t="n"/>
@@ -20697,8 +20798,15 @@
       <c r="D37" s="19" t="n"/>
       <c r="E37" s="19" t="n"/>
     </row>
+    <row r="38">
+      <c r="A38" s="19" t="n"/>
+      <c r="B38" s="19" t="n"/>
+      <c r="C38" s="19" t="n"/>
+      <c r="D38" s="19" t="n"/>
+      <c r="E38" s="19" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:E35"/>
+  <autoFilter ref="A8:E36"/>
   <mergeCells count="6">
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
@@ -20717,7 +20825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -20775,26 +20883,33 @@
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>Brecha: coexisten el criterio de media del bloque (MSAVI &lt; 0.4976) y el criterio areal del E6; no son sumables entre sí.</t>
+          <t>Brecha: coexisten el criterio de media del bloque (MSAVI &lt; 0.4976), el criterio areal del E6 y la media del MSAVI por ecosistema que propone el Plan de Trabajo institucional v2; no son sumables entre sí.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>Situación predial de gabinete: superficie sin registro en GEORURAL y COFOPRI se asume Tierras del Estado y/o posesionarios; requiere verificación de campo y actas.</t>
+          <t>E6: se desarrolla con la metodología de firma espectral por el equipo base, conforme al Plan de Trabajo Detallado – Actualización N° 01, Versión 2 (16/10/2026); las observaciones OE-03 y OE-14 a OE-16 alinean el Informe E6 y las matrices con dicho plan.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>Los totales de cada hoja se calculan con fórmulas (=SUM, =COUNTA) sobre las filas de la tabla.</t>
+          <t>Situación predial de gabinete: superficie sin registro en GEORURAL y COFOPRI se asume Tierras del Estado y/o posesionarios; requiere verificación de campo y actas.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Los totales de cada hoja se calculan con fórmulas (=SUM, =COUNTA) sobre las filas de la tabla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>Las observaciones al Estudio de Suelos y al E6 se levantan en los entregables indicados; su estado corresponde al corte del Segundo Entregable.</t>
         </is>

</xml_diff>